<commit_message>
feat: 003 上传批次 UP-20260417-162837
- mode: local-copy
- target: github_pages
- state: Excel + upload_state.json + upload log
</commit_message>
<xml_diff>
--- a/assets/products/产品识别.xlsx
+++ b/assets/products/产品识别.xlsx
@@ -1097,7 +1097,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R20"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="0"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -1244,7 +1244,11 @@
           <t>否</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>PRD-UNKNOWN-2</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>003_已回写</t>
@@ -1267,28 +1271,28 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17 16:00:32</t>
+          <t>2026-04-17 16:10:01</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>github_pages</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>UP-20260417-160032</t>
+          <t>UP-20260417-161001</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>模拟上传成功</t>
+          <t>人工确认已上传: IK200101-A-16-1-7.jpg -&gt; manual</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17 16:00:32</t>
+          <t>2026-04-17 16:10:01</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1329,11 @@
           <t>否</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>PRD-UNKNOWN-3</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>003_已回写</t>
@@ -1348,28 +1356,28 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17 16:00:32</t>
+          <t>2026-04-17 16:10:01</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>github_pages</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>UP-20260417-160032</t>
+          <t>UP-20260417-161001</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>模拟上传成功</t>
+          <t>人工确认已上传: IK2036-A-16-mian01.jpg -&gt; manual</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17 16:00:32</t>
+          <t>2026-04-17 16:10:01</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1414,11 @@
           <t>否</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>PRD-UNKNOWN-4</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>003_已回写</t>
@@ -1429,28 +1441,28 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17 16:00:32</t>
+          <t>2026-04-17 16:21:03</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>github_pages</t>
+          <t>local_outbox</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>UP-20260417-160032</t>
+          <t>UP-20260417-162103</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>模拟上传成功</t>
+          <t>已复制到 003 上传目录: C:\Users\Win11\Desktop\XCSOURCE\assets\products\uploaded_by_003\UP-20260417-162103\PRD-UNKNOWN-4\IK500302-A-16-1-2.jpg</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17 16:00:32</t>
+          <t>2026-04-17 16:21:03</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1499,11 @@
           <t>否</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>PRD-UNKNOWN-5</t>
+        </is>
+      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>003_已回写</t>
@@ -1510,7 +1526,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17 16:00:32</t>
+          <t>2026-04-17 16:28:37</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1520,18 +1536,18 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>UP-20260417-160032</t>
+          <t>UP-20260417-162837</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>模拟上传成功</t>
+          <t>已复制到 003 上传目录: C:\Users\Win11\Desktop\XCSOURCE\assets\products\uploaded_by_003\UP-20260417-162837\PRD-UNKNOWN-5\IK600209-A-16-1-1.jpg</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17 16:00:32</t>
+          <t>2026-04-17 16:28:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: 003 上传批次 UP-20260417-163632
- mode: local-copy
- target: github_pages
- state: Excel + upload_state.json + upload log + manifest
</commit_message>
<xml_diff>
--- a/assets/products/产品识别.xlsx
+++ b/assets/products/产品识别.xlsx
@@ -1584,7 +1584,11 @@
           <t>否</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>PRD-UNKNOWN-6</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>003_已回写</t>
@@ -1607,7 +1611,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17 16:00:32</t>
+          <t>2026-04-17 16:36:32</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -1617,18 +1621,18 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>UP-20260417-160032</t>
+          <t>UP-20260417-163632</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>模拟上传成功</t>
+          <t>已复制到 003 上传目录: C:\Users\Win11\Desktop\XCSOURCE\assets\products\uploaded_by_003\UP-20260417-163632\PRD-UNKNOWN-6\IK800301-A-16-1-1.jpg</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17 16:00:32</t>
+          <t>2026-04-17 16:36:32</t>
         </is>
       </c>
     </row>

</xml_diff>